<commit_message>
feat(S7): generate a strategy driver from a flow spec wiring the callbacks; S8 cross-checks flow vs execution steps and dry-runs it; 大小周期共振 regenerated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workspace/大小周期共振/S7_formal.xlsx
+++ b/workspace/大小周期共振/S7_formal.xlsx
@@ -10,7 +10,8 @@
     <sheet name="callbacks" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="parameters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="relations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="legend" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="flow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="legend" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1962,7 +1963,447 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>when</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>call</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bind</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>args</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>when_result</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>then</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>next</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>step_ref</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>note_en</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>note_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CB01</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.1</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>每次评估先刷新大周期方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>direction in ('long', 'short')</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>CB02</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>{"major_direction": "direction"}</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.2</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>只在方向明确时评估同向入场信号</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>F03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>entry is not None and entry.decision == 'enter'</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CB03</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>{"entry_price": "entry.entry_price"}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>enter</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>IN_POSITION</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.3</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>入场并按小周期止损设初始止损；此后只看大周期</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>IN_POSITION</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>stop_hit</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>close:stop</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>exit_and_risk.4</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>出场路径一：打止损</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>IN_POSITION</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>CB05</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>reversed</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>{"major_direction": "direction"}</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>reversed</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>close:reversal</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.5</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>出场路径二：大周期趋势反转主动清仓</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>IN_POSITION</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>not position.stop_at_cost</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CB06</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>favorable</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>favorable</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>move_stop_to_cost</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.4</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>有利运动后尽快移损至成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>F07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>IN_POSITION</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>position.stop_at_cost</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>CB04</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>new_stop</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>new_stop is not None</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>move_stop</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>execution_steps.5</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>移损至成本后按大周期信号移动止损，只进不退</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2073,13 +2514,30 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>flow.*</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>one rule per row; see references/flow_dsl.md; args is a JSON object</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>每行一条控制流规则，见 references/flow_dsl.md；args 为 JSON 对象</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>Agents read the json; edit here then run sf_formal.py from-xlsx.</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>供人编辑，改完运行 from-xlsx</t>
         </is>

</xml_diff>